<commit_message>
Final Measurements for Multi-Tenant use
</commit_message>
<xml_diff>
--- a/results/GEMV_Chart_Data.xlsx
+++ b/results/GEMV_Chart_Data.xlsx
@@ -24,6 +24,12 @@
     <sheet name="Family Utilization" sheetId="15" state="visible" r:id="rId15"/>
     <sheet name="Family Mixed Latency" sheetId="16" state="visible" r:id="rId16"/>
     <sheet name="Family Mixed Energy" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet name="MT Interference" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet name="MT Throughput" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet name="MT Energy" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet name="Scale-out vs Scale-up" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet name="Idle vs Channels" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet name="Configurations" sheetId="23" state="visible" r:id="rId23"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'avg3 comparison'!$A$1:$AH$13</definedName>
@@ -43,6 +49,12 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="14" hidden="1">'Family Utilization'!$A$1:$V$7</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="15" hidden="1">'Family Mixed Latency'!$A$1:$S$12</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="16" hidden="1">'Family Mixed Energy'!$A$1:$W$67</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="17" hidden="1">'MT Interference'!$A$1:$S$9</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="18" hidden="1">'MT Throughput'!$A$1:$M$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="19" hidden="1">'MT Energy'!$A$1:$Q$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="20" hidden="1">'Scale-out vs Scale-up'!$A$1:$H$7</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="21" hidden="1">'Idle vs Channels'!$A$1:$K$14</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="22" hidden="1">'Configurations'!$A$1:$AC$14</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -16807,6 +16819,921 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:S9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="17" customWidth="1" min="2" max="2"/>
+    <col width="17" customWidth="1" min="3" max="3"/>
+    <col width="17" customWidth="1" min="4" max="4"/>
+    <col width="17" customWidth="1" min="5" max="5"/>
+    <col width="17" customWidth="1" min="6" max="6"/>
+    <col width="17" customWidth="1" min="7" max="7"/>
+    <col width="17" customWidth="1" min="8" max="8"/>
+    <col width="17" customWidth="1" min="9" max="9"/>
+    <col width="17" customWidth="1" min="10" max="10"/>
+    <col width="17" customWidth="1" min="11" max="11"/>
+    <col width="17" customWidth="1" min="12" max="12"/>
+    <col width="20" customWidth="1" min="13" max="13"/>
+    <col width="22" customWidth="1" min="14" max="14"/>
+    <col width="15" customWidth="1" min="15" max="15"/>
+    <col width="11" customWidth="1" min="16" max="16"/>
+    <col width="30" customWidth="1" min="17" max="17"/>
+    <col width="11" customWidth="1" min="18" max="18"/>
+    <col width="30" customWidth="1" min="19" max="19"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>workload</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>tenants_running</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>slowdown_pct_t0</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>slowdown_pct_t1</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>slowdown_pct_t2</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>slowdown_pct_t3</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>slowdown_pct_t4</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>interference_t0</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>interference_t1</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>interference_t2</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>interference_t3</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>interference_t4</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>active_overlap_pct</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>alone_spread_pct_max</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>workload_name</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>tenants_n</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>bitstream</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>clock_mhz</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>estimator</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>2 tenants</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="n">
+        <v>0.89</v>
+      </c>
+      <c r="D2" s="2" t="n">
+        <v>-1.07</v>
+      </c>
+      <c r="H2" s="2" t="n">
+        <v>1.0089</v>
+      </c>
+      <c r="I2" s="2" t="n">
+        <v>0.9893</v>
+      </c>
+      <c r="M2" s="2" t="n">
+        <v>97.37</v>
+      </c>
+      <c r="N2" s="2" t="n">
+        <v>0.994</v>
+      </c>
+      <c r="O2" s="2" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+      <c r="P2" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q2" s="2" t="inlineStr">
+        <is>
+          <t>sparse_4x4_x5_375_split.xclbin</t>
+        </is>
+      </c>
+      <c r="R2" s="2" t="n">
+        <v>329</v>
+      </c>
+      <c r="S2" s="2" t="inlineStr">
+        <is>
+          <t>active-span ratio vs the same tenant alone, mean of 3 reps</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>3 tenants</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="n">
+        <v>0.97</v>
+      </c>
+      <c r="D3" s="2" t="n">
+        <v>-0.66</v>
+      </c>
+      <c r="E3" s="2" t="n">
+        <v>-0.37</v>
+      </c>
+      <c r="H3" s="2" t="n">
+        <v>1.0097</v>
+      </c>
+      <c r="I3" s="2" t="n">
+        <v>0.9933999999999999</v>
+      </c>
+      <c r="J3" s="2" t="n">
+        <v>0.9963</v>
+      </c>
+      <c r="M3" s="2" t="n">
+        <v>94.27</v>
+      </c>
+      <c r="N3" s="2" t="n">
+        <v>0.994</v>
+      </c>
+      <c r="O3" s="2" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+      <c r="P3" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q3" s="2" t="inlineStr">
+        <is>
+          <t>sparse_4x4_x5_375_split.xclbin</t>
+        </is>
+      </c>
+      <c r="R3" s="2" t="n">
+        <v>329</v>
+      </c>
+      <c r="S3" s="2" t="inlineStr">
+        <is>
+          <t>active-span ratio vs the same tenant alone, mean of 3 reps</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>4 tenants</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="n">
+        <v>1.18</v>
+      </c>
+      <c r="D4" s="2" t="n">
+        <v>-0.14</v>
+      </c>
+      <c r="E4" s="2" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="F4" s="2" t="n">
+        <v>-0.3</v>
+      </c>
+      <c r="H4" s="2" t="n">
+        <v>1.0118</v>
+      </c>
+      <c r="I4" s="2" t="n">
+        <v>0.9986</v>
+      </c>
+      <c r="J4" s="2" t="n">
+        <v>1.0005</v>
+      </c>
+      <c r="K4" s="2" t="n">
+        <v>0.997</v>
+      </c>
+      <c r="M4" s="2" t="n">
+        <v>91.5</v>
+      </c>
+      <c r="N4" s="2" t="n">
+        <v>0.994</v>
+      </c>
+      <c r="O4" s="2" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+      <c r="P4" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="Q4" s="2" t="inlineStr">
+        <is>
+          <t>sparse_4x4_x5_375_split.xclbin</t>
+        </is>
+      </c>
+      <c r="R4" s="2" t="n">
+        <v>329</v>
+      </c>
+      <c r="S4" s="2" t="inlineStr">
+        <is>
+          <t>active-span ratio vs the same tenant alone, mean of 3 reps</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>5 tenants</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="n">
+        <v>1.45</v>
+      </c>
+      <c r="D5" s="2" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="E5" s="2" t="n">
+        <v>0.46</v>
+      </c>
+      <c r="F5" s="2" t="n">
+        <v>-0.38</v>
+      </c>
+      <c r="G5" s="2" t="n">
+        <v>-0.28</v>
+      </c>
+      <c r="H5" s="2" t="n">
+        <v>1.0145</v>
+      </c>
+      <c r="I5" s="2" t="n">
+        <v>1.0004</v>
+      </c>
+      <c r="J5" s="2" t="n">
+        <v>1.0046</v>
+      </c>
+      <c r="K5" s="2" t="n">
+        <v>0.9962</v>
+      </c>
+      <c r="L5" s="2" t="n">
+        <v>0.9972</v>
+      </c>
+      <c r="M5" s="2" t="n">
+        <v>88.27</v>
+      </c>
+      <c r="N5" s="2" t="n">
+        <v>0.994</v>
+      </c>
+      <c r="O5" s="2" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+      <c r="P5" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="Q5" s="2" t="inlineStr">
+        <is>
+          <t>sparse_4x4_x5_375_split.xclbin</t>
+        </is>
+      </c>
+      <c r="R5" s="2" t="n">
+        <v>329</v>
+      </c>
+      <c r="S5" s="2" t="inlineStr">
+        <is>
+          <t>active-span ratio vs the same tenant alone, mean of 3 reps</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>All 2:32</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>2 tenants</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="n">
+        <v>0.43</v>
+      </c>
+      <c r="D6" s="2" t="n">
+        <v>-0.8</v>
+      </c>
+      <c r="H6" s="2" t="n">
+        <v>1.0043</v>
+      </c>
+      <c r="I6" s="2" t="n">
+        <v>0.992</v>
+      </c>
+      <c r="M6" s="2" t="n">
+        <v>95.56999999999999</v>
+      </c>
+      <c r="N6" s="2" t="n">
+        <v>0.441</v>
+      </c>
+      <c r="O6" s="2" t="inlineStr">
+        <is>
+          <t>All 2:32</t>
+        </is>
+      </c>
+      <c r="P6" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q6" s="2" t="inlineStr">
+        <is>
+          <t>sparse_4x4_x5_375_split.xclbin</t>
+        </is>
+      </c>
+      <c r="R6" s="2" t="n">
+        <v>329</v>
+      </c>
+      <c r="S6" s="2" t="inlineStr">
+        <is>
+          <t>active-span ratio vs the same tenant alone, mean of 3 reps</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>3 tenants</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="n">
+        <v>0.39</v>
+      </c>
+      <c r="D7" s="2" t="n">
+        <v>-0.8</v>
+      </c>
+      <c r="E7" s="2" t="n">
+        <v>-0.08</v>
+      </c>
+      <c r="H7" s="2" t="n">
+        <v>1.0039</v>
+      </c>
+      <c r="I7" s="2" t="n">
+        <v>0.992</v>
+      </c>
+      <c r="J7" s="2" t="n">
+        <v>0.9992</v>
+      </c>
+      <c r="M7" s="2" t="n">
+        <v>92.06999999999999</v>
+      </c>
+      <c r="N7" s="2" t="n">
+        <v>0.441</v>
+      </c>
+      <c r="O7" s="2" t="inlineStr">
+        <is>
+          <t>All 2:32</t>
+        </is>
+      </c>
+      <c r="P7" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q7" s="2" t="inlineStr">
+        <is>
+          <t>sparse_4x4_x5_375_split.xclbin</t>
+        </is>
+      </c>
+      <c r="R7" s="2" t="n">
+        <v>329</v>
+      </c>
+      <c r="S7" s="2" t="inlineStr">
+        <is>
+          <t>active-span ratio vs the same tenant alone, mean of 3 reps</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>4 tenants</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="n">
+        <v>0.41</v>
+      </c>
+      <c r="D8" s="2" t="n">
+        <v>-0.64</v>
+      </c>
+      <c r="E8" s="2" t="n">
+        <v>0.13</v>
+      </c>
+      <c r="F8" s="2" t="n">
+        <v>-0.41</v>
+      </c>
+      <c r="H8" s="2" t="n">
+        <v>1.0041</v>
+      </c>
+      <c r="I8" s="2" t="n">
+        <v>0.9936</v>
+      </c>
+      <c r="J8" s="2" t="n">
+        <v>1.0013</v>
+      </c>
+      <c r="K8" s="2" t="n">
+        <v>0.9959</v>
+      </c>
+      <c r="M8" s="2" t="n">
+        <v>85.03</v>
+      </c>
+      <c r="N8" s="2" t="n">
+        <v>0.441</v>
+      </c>
+      <c r="O8" s="2" t="inlineStr">
+        <is>
+          <t>All 2:32</t>
+        </is>
+      </c>
+      <c r="P8" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="Q8" s="2" t="inlineStr">
+        <is>
+          <t>sparse_4x4_x5_375_split.xclbin</t>
+        </is>
+      </c>
+      <c r="R8" s="2" t="n">
+        <v>329</v>
+      </c>
+      <c r="S8" s="2" t="inlineStr">
+        <is>
+          <t>active-span ratio vs the same tenant alone, mean of 3 reps</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>5 tenants</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="n">
+        <v>0.92</v>
+      </c>
+      <c r="D9" s="2" t="n">
+        <v>-0.06</v>
+      </c>
+      <c r="E9" s="2" t="n">
+        <v>0.46</v>
+      </c>
+      <c r="F9" s="2" t="n">
+        <v>-0.62</v>
+      </c>
+      <c r="G9" s="2" t="n">
+        <v>-0.01</v>
+      </c>
+      <c r="H9" s="2" t="n">
+        <v>1.0092</v>
+      </c>
+      <c r="I9" s="2" t="n">
+        <v>0.9994</v>
+      </c>
+      <c r="J9" s="2" t="n">
+        <v>1.0046</v>
+      </c>
+      <c r="K9" s="2" t="n">
+        <v>0.9938</v>
+      </c>
+      <c r="L9" s="2" t="n">
+        <v>0.9999</v>
+      </c>
+      <c r="M9" s="2" t="n">
+        <v>83.90000000000001</v>
+      </c>
+      <c r="N9" s="2" t="n">
+        <v>0.441</v>
+      </c>
+      <c r="O9" s="2" t="inlineStr">
+        <is>
+          <t>All 2:32</t>
+        </is>
+      </c>
+      <c r="P9" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="Q9" s="2" t="inlineStr">
+        <is>
+          <t>sparse_4x4_x5_375_split.xclbin</t>
+        </is>
+      </c>
+      <c r="R9" s="2" t="n">
+        <v>329</v>
+      </c>
+      <c r="S9" s="2" t="inlineStr">
+        <is>
+          <t>active-span ratio vs the same tenant alone, mean of 3 reps</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:S9"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:M6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="17" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="17" customWidth="1" min="3" max="3"/>
+    <col width="23" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="17" customWidth="1" min="6" max="6"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
+    <col width="19" customWidth="1" min="8" max="8"/>
+    <col width="22" customWidth="1" min="9" max="9"/>
+    <col width="11" customWidth="1" min="10" max="10"/>
+    <col width="30" customWidth="1" min="11" max="11"/>
+    <col width="11" customWidth="1" min="12" max="12"/>
+    <col width="30" customWidth="1" min="13" max="13"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>tenants_running</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>gmac_s_mixed</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>gmac_s_all2to32</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>gmac_s_linear_scaling</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>gmac_s_peak</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>scaling_x_mixed</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>scaling_x_all2to32</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>pct_of_peak_mixed</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>pct_of_peak_all2to32</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>tenants_n</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>bitstream</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>clock_mhz</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>estimator</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>1 tenant</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="n">
+        <v>9.881</v>
+      </c>
+      <c r="C2" s="2" t="n">
+        <v>9.728999999999999</v>
+      </c>
+      <c r="D2" s="2" t="n">
+        <v>9.881</v>
+      </c>
+      <c r="E2" s="2" t="n">
+        <v>10.528</v>
+      </c>
+      <c r="F2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H2" s="2" t="n">
+        <v>93.84999999999999</v>
+      </c>
+      <c r="I2" s="2" t="n">
+        <v>92.41</v>
+      </c>
+      <c r="J2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>sparse_4x4_x5_375_split.xclbin</t>
+        </is>
+      </c>
+      <c r="L2" s="2" t="n">
+        <v>329</v>
+      </c>
+      <c r="M2" s="2" t="inlineStr">
+        <is>
+          <t>60 s power soak, host calculation counts x MACs per calculation</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>2 tenants</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="n">
+        <v>19.743</v>
+      </c>
+      <c r="C3" s="2" t="n">
+        <v>19.13</v>
+      </c>
+      <c r="D3" s="2" t="n">
+        <v>19.762</v>
+      </c>
+      <c r="E3" s="2" t="n">
+        <v>21.056</v>
+      </c>
+      <c r="F3" s="2" t="n">
+        <v>1.998</v>
+      </c>
+      <c r="G3" s="2" t="n">
+        <v>1.966</v>
+      </c>
+      <c r="H3" s="2" t="n">
+        <v>93.76000000000001</v>
+      </c>
+      <c r="I3" s="2" t="n">
+        <v>90.84999999999999</v>
+      </c>
+      <c r="J3" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>sparse_4x4_x5_375_split.xclbin</t>
+        </is>
+      </c>
+      <c r="L3" s="2" t="n">
+        <v>329</v>
+      </c>
+      <c r="M3" s="2" t="inlineStr">
+        <is>
+          <t>60 s power soak, host calculation counts x MACs per calculation</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>3 tenants</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="n">
+        <v>29.351</v>
+      </c>
+      <c r="C4" s="2" t="n">
+        <v>28.938</v>
+      </c>
+      <c r="D4" s="2" t="n">
+        <v>29.643</v>
+      </c>
+      <c r="E4" s="2" t="n">
+        <v>31.584</v>
+      </c>
+      <c r="F4" s="2" t="n">
+        <v>2.97</v>
+      </c>
+      <c r="G4" s="2" t="n">
+        <v>2.974</v>
+      </c>
+      <c r="H4" s="2" t="n">
+        <v>92.93000000000001</v>
+      </c>
+      <c r="I4" s="2" t="n">
+        <v>91.62</v>
+      </c>
+      <c r="J4" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="K4" s="2" t="inlineStr">
+        <is>
+          <t>sparse_4x4_x5_375_split.xclbin</t>
+        </is>
+      </c>
+      <c r="L4" s="2" t="n">
+        <v>329</v>
+      </c>
+      <c r="M4" s="2" t="inlineStr">
+        <is>
+          <t>60 s power soak, host calculation counts x MACs per calculation</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>4 tenants</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="n">
+        <v>39.196</v>
+      </c>
+      <c r="C5" s="2" t="n">
+        <v>37.706</v>
+      </c>
+      <c r="D5" s="2" t="n">
+        <v>39.524</v>
+      </c>
+      <c r="E5" s="2" t="n">
+        <v>42.112</v>
+      </c>
+      <c r="F5" s="2" t="n">
+        <v>3.967</v>
+      </c>
+      <c r="G5" s="2" t="n">
+        <v>3.876</v>
+      </c>
+      <c r="H5" s="2" t="n">
+        <v>93.08</v>
+      </c>
+      <c r="I5" s="2" t="n">
+        <v>89.54000000000001</v>
+      </c>
+      <c r="J5" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="K5" s="2" t="inlineStr">
+        <is>
+          <t>sparse_4x4_x5_375_split.xclbin</t>
+        </is>
+      </c>
+      <c r="L5" s="2" t="n">
+        <v>329</v>
+      </c>
+      <c r="M5" s="2" t="inlineStr">
+        <is>
+          <t>60 s power soak, host calculation counts x MACs per calculation</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>5 tenants</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="n">
+        <v>48.543</v>
+      </c>
+      <c r="C6" s="2" t="n">
+        <v>47.209</v>
+      </c>
+      <c r="D6" s="2" t="n">
+        <v>49.405</v>
+      </c>
+      <c r="E6" s="2" t="n">
+        <v>52.64</v>
+      </c>
+      <c r="F6" s="2" t="n">
+        <v>4.913</v>
+      </c>
+      <c r="G6" s="2" t="n">
+        <v>4.852</v>
+      </c>
+      <c r="H6" s="2" t="n">
+        <v>92.22</v>
+      </c>
+      <c r="I6" s="2" t="n">
+        <v>89.68000000000001</v>
+      </c>
+      <c r="J6" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="K6" s="2" t="inlineStr">
+        <is>
+          <t>sparse_4x4_x5_375_split.xclbin</t>
+        </is>
+      </c>
+      <c r="L6" s="2" t="n">
+        <v>329</v>
+      </c>
+      <c r="M6" s="2" t="inlineStr">
+        <is>
+          <t>60 s power soak, host calculation counts x MACs per calculation</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:M6"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
@@ -17674,6 +18601,3033 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:AH7"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:Q11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="17" customWidth="1" min="2" max="2"/>
+    <col width="19" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="17" customWidth="1" min="9" max="9"/>
+    <col width="15" customWidth="1" min="10" max="10"/>
+    <col width="15" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="15" customWidth="1" min="13" max="13"/>
+    <col width="11" customWidth="1" min="14" max="14"/>
+    <col width="30" customWidth="1" min="15" max="15"/>
+    <col width="11" customWidth="1" min="16" max="16"/>
+    <col width="30" customWidth="1" min="17" max="17"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>workload</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>tenants_running</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>static_nJ_per_MAC</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>dynamic_nJ_per_MAC</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>total_nJ_per_MAC</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>gmac_s</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>board_load_W</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>board_idle_W</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>board_dynamic_W</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>vccint_load_W</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>vccint_idle_W</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>static_pct</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>workload_name</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>tenants_n</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>bitstream</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>clock_mhz</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>estimator</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>1 tenant</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="n">
+        <v>3.4154</v>
+      </c>
+      <c r="D2" s="2" t="n">
+        <v>0.1598</v>
+      </c>
+      <c r="E2" s="2" t="n">
+        <v>3.5752</v>
+      </c>
+      <c r="F2" s="2" t="n">
+        <v>9.881</v>
+      </c>
+      <c r="G2" s="2" t="n">
+        <v>35.327</v>
+      </c>
+      <c r="H2" s="2" t="n">
+        <v>33.748</v>
+      </c>
+      <c r="I2" s="2" t="n">
+        <v>1.579</v>
+      </c>
+      <c r="J2" s="2" t="n">
+        <v>9.077</v>
+      </c>
+      <c r="K2" s="2" t="n">
+        <v>8.705</v>
+      </c>
+      <c r="L2" s="2" t="n">
+        <v>95.53</v>
+      </c>
+      <c r="M2" s="2" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+      <c r="N2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="O2" s="2" t="inlineStr">
+        <is>
+          <t>sparse_4x4_x5_375_split.xclbin</t>
+        </is>
+      </c>
+      <c r="P2" s="2" t="n">
+        <v>329</v>
+      </c>
+      <c r="Q2" s="2" t="inlineStr">
+        <is>
+          <t>60 s power soak, host calculation counts x MACs per calculation; static = idle after the soak, dynamic = load - idle</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>2 tenants</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="n">
+        <v>1.7125</v>
+      </c>
+      <c r="D3" s="2" t="n">
+        <v>0.1619</v>
+      </c>
+      <c r="E3" s="2" t="n">
+        <v>1.8744</v>
+      </c>
+      <c r="F3" s="2" t="n">
+        <v>19.743</v>
+      </c>
+      <c r="G3" s="2" t="n">
+        <v>37.005</v>
+      </c>
+      <c r="H3" s="2" t="n">
+        <v>33.809</v>
+      </c>
+      <c r="I3" s="2" t="n">
+        <v>3.196</v>
+      </c>
+      <c r="J3" s="2" t="n">
+        <v>9.342000000000001</v>
+      </c>
+      <c r="K3" s="2" t="n">
+        <v>8.702999999999999</v>
+      </c>
+      <c r="L3" s="2" t="n">
+        <v>91.36</v>
+      </c>
+      <c r="M3" s="2" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+      <c r="N3" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="O3" s="2" t="inlineStr">
+        <is>
+          <t>sparse_4x4_x5_375_split.xclbin</t>
+        </is>
+      </c>
+      <c r="P3" s="2" t="n">
+        <v>329</v>
+      </c>
+      <c r="Q3" s="2" t="inlineStr">
+        <is>
+          <t>60 s power soak, host calculation counts x MACs per calculation; static = idle after the soak, dynamic = load - idle</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>3 tenants</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="n">
+        <v>1.1517</v>
+      </c>
+      <c r="D4" s="2" t="n">
+        <v>0.1661</v>
+      </c>
+      <c r="E4" s="2" t="n">
+        <v>1.3177</v>
+      </c>
+      <c r="F4" s="2" t="n">
+        <v>29.351</v>
+      </c>
+      <c r="G4" s="2" t="n">
+        <v>38.676</v>
+      </c>
+      <c r="H4" s="2" t="n">
+        <v>33.802</v>
+      </c>
+      <c r="I4" s="2" t="n">
+        <v>4.874</v>
+      </c>
+      <c r="J4" s="2" t="n">
+        <v>9.67</v>
+      </c>
+      <c r="K4" s="2" t="n">
+        <v>8.699</v>
+      </c>
+      <c r="L4" s="2" t="n">
+        <v>87.40000000000001</v>
+      </c>
+      <c r="M4" s="2" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+      <c r="N4" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="O4" s="2" t="inlineStr">
+        <is>
+          <t>sparse_4x4_x5_375_split.xclbin</t>
+        </is>
+      </c>
+      <c r="P4" s="2" t="n">
+        <v>329</v>
+      </c>
+      <c r="Q4" s="2" t="inlineStr">
+        <is>
+          <t>60 s power soak, host calculation counts x MACs per calculation; static = idle after the soak, dynamic = load - idle</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>4 tenants</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="n">
+        <v>0.8641</v>
+      </c>
+      <c r="D5" s="2" t="n">
+        <v>0.1646</v>
+      </c>
+      <c r="E5" s="2" t="n">
+        <v>1.0287</v>
+      </c>
+      <c r="F5" s="2" t="n">
+        <v>39.196</v>
+      </c>
+      <c r="G5" s="2" t="n">
+        <v>40.321</v>
+      </c>
+      <c r="H5" s="2" t="n">
+        <v>33.87</v>
+      </c>
+      <c r="I5" s="2" t="n">
+        <v>6.451</v>
+      </c>
+      <c r="J5" s="2" t="n">
+        <v>10.018</v>
+      </c>
+      <c r="K5" s="2" t="n">
+        <v>8.852</v>
+      </c>
+      <c r="L5" s="2" t="n">
+        <v>84</v>
+      </c>
+      <c r="M5" s="2" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+      <c r="N5" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="O5" s="2" t="inlineStr">
+        <is>
+          <t>sparse_4x4_x5_375_split.xclbin</t>
+        </is>
+      </c>
+      <c r="P5" s="2" t="n">
+        <v>329</v>
+      </c>
+      <c r="Q5" s="2" t="inlineStr">
+        <is>
+          <t>60 s power soak, host calculation counts x MACs per calculation; static = idle after the soak, dynamic = load - idle</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>5 tenants</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="n">
+        <v>0.6956</v>
+      </c>
+      <c r="D6" s="2" t="n">
+        <v>0.1734</v>
+      </c>
+      <c r="E6" s="2" t="n">
+        <v>0.8691</v>
+      </c>
+      <c r="F6" s="2" t="n">
+        <v>48.543</v>
+      </c>
+      <c r="G6" s="2" t="n">
+        <v>42.187</v>
+      </c>
+      <c r="H6" s="2" t="n">
+        <v>33.768</v>
+      </c>
+      <c r="I6" s="2" t="n">
+        <v>8.419</v>
+      </c>
+      <c r="J6" s="2" t="n">
+        <v>10.465</v>
+      </c>
+      <c r="K6" s="2" t="n">
+        <v>8.835000000000001</v>
+      </c>
+      <c r="L6" s="2" t="n">
+        <v>80.04000000000001</v>
+      </c>
+      <c r="M6" s="2" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+      <c r="N6" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="O6" s="2" t="inlineStr">
+        <is>
+          <t>sparse_4x4_x5_375_split.xclbin</t>
+        </is>
+      </c>
+      <c r="P6" s="2" t="n">
+        <v>329</v>
+      </c>
+      <c r="Q6" s="2" t="inlineStr">
+        <is>
+          <t>60 s power soak, host calculation counts x MACs per calculation; static = idle after the soak, dynamic = load - idle</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>All 2:32</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>1 tenant</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="n">
+        <v>3.4537</v>
+      </c>
+      <c r="D7" s="2" t="n">
+        <v>0.1738</v>
+      </c>
+      <c r="E7" s="2" t="n">
+        <v>3.6275</v>
+      </c>
+      <c r="F7" s="2" t="n">
+        <v>9.728999999999999</v>
+      </c>
+      <c r="G7" s="2" t="n">
+        <v>35.293</v>
+      </c>
+      <c r="H7" s="2" t="n">
+        <v>33.602</v>
+      </c>
+      <c r="I7" s="2" t="n">
+        <v>1.691</v>
+      </c>
+      <c r="J7" s="2" t="n">
+        <v>8.970000000000001</v>
+      </c>
+      <c r="K7" s="2" t="n">
+        <v>8.525</v>
+      </c>
+      <c r="L7" s="2" t="n">
+        <v>95.20999999999999</v>
+      </c>
+      <c r="M7" s="2" t="inlineStr">
+        <is>
+          <t>All 2:32</t>
+        </is>
+      </c>
+      <c r="N7" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="O7" s="2" t="inlineStr">
+        <is>
+          <t>sparse_4x4_x5_375_split.xclbin</t>
+        </is>
+      </c>
+      <c r="P7" s="2" t="n">
+        <v>329</v>
+      </c>
+      <c r="Q7" s="2" t="inlineStr">
+        <is>
+          <t>60 s power soak, host calculation counts x MACs per calculation; static = idle after the soak, dynamic = load - idle</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>2 tenants</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="n">
+        <v>1.7479</v>
+      </c>
+      <c r="D8" s="2" t="n">
+        <v>0.1741</v>
+      </c>
+      <c r="E8" s="2" t="n">
+        <v>1.922</v>
+      </c>
+      <c r="F8" s="2" t="n">
+        <v>19.13</v>
+      </c>
+      <c r="G8" s="2" t="n">
+        <v>36.767</v>
+      </c>
+      <c r="H8" s="2" t="n">
+        <v>33.437</v>
+      </c>
+      <c r="I8" s="2" t="n">
+        <v>3.33</v>
+      </c>
+      <c r="J8" s="2" t="n">
+        <v>9.193</v>
+      </c>
+      <c r="K8" s="2" t="n">
+        <v>8.522</v>
+      </c>
+      <c r="L8" s="2" t="n">
+        <v>90.94</v>
+      </c>
+      <c r="M8" s="2" t="inlineStr">
+        <is>
+          <t>All 2:32</t>
+        </is>
+      </c>
+      <c r="N8" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="O8" s="2" t="inlineStr">
+        <is>
+          <t>sparse_4x4_x5_375_split.xclbin</t>
+        </is>
+      </c>
+      <c r="P8" s="2" t="n">
+        <v>329</v>
+      </c>
+      <c r="Q8" s="2" t="inlineStr">
+        <is>
+          <t>60 s power soak, host calculation counts x MACs per calculation; static = idle after the soak, dynamic = load - idle</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>3 tenants</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="n">
+        <v>1.1588</v>
+      </c>
+      <c r="D9" s="2" t="n">
+        <v>0.1713</v>
+      </c>
+      <c r="E9" s="2" t="n">
+        <v>1.3301</v>
+      </c>
+      <c r="F9" s="2" t="n">
+        <v>28.938</v>
+      </c>
+      <c r="G9" s="2" t="n">
+        <v>38.49</v>
+      </c>
+      <c r="H9" s="2" t="n">
+        <v>33.532</v>
+      </c>
+      <c r="I9" s="2" t="n">
+        <v>4.958</v>
+      </c>
+      <c r="J9" s="2" t="n">
+        <v>9.539</v>
+      </c>
+      <c r="K9" s="2" t="n">
+        <v>8.516</v>
+      </c>
+      <c r="L9" s="2" t="n">
+        <v>87.12</v>
+      </c>
+      <c r="M9" s="2" t="inlineStr">
+        <is>
+          <t>All 2:32</t>
+        </is>
+      </c>
+      <c r="N9" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="O9" s="2" t="inlineStr">
+        <is>
+          <t>sparse_4x4_x5_375_split.xclbin</t>
+        </is>
+      </c>
+      <c r="P9" s="2" t="n">
+        <v>329</v>
+      </c>
+      <c r="Q9" s="2" t="inlineStr">
+        <is>
+          <t>60 s power soak, host calculation counts x MACs per calculation; static = idle after the soak, dynamic = load - idle</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>4 tenants</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="n">
+        <v>0.8874</v>
+      </c>
+      <c r="D10" s="2" t="n">
+        <v>0.1756</v>
+      </c>
+      <c r="E10" s="2" t="n">
+        <v>1.063</v>
+      </c>
+      <c r="F10" s="2" t="n">
+        <v>37.706</v>
+      </c>
+      <c r="G10" s="2" t="n">
+        <v>40.083</v>
+      </c>
+      <c r="H10" s="2" t="n">
+        <v>33.461</v>
+      </c>
+      <c r="I10" s="2" t="n">
+        <v>6.622</v>
+      </c>
+      <c r="J10" s="2" t="n">
+        <v>9.891999999999999</v>
+      </c>
+      <c r="K10" s="2" t="n">
+        <v>8.521000000000001</v>
+      </c>
+      <c r="L10" s="2" t="n">
+        <v>83.48</v>
+      </c>
+      <c r="M10" s="2" t="inlineStr">
+        <is>
+          <t>All 2:32</t>
+        </is>
+      </c>
+      <c r="N10" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="O10" s="2" t="inlineStr">
+        <is>
+          <t>sparse_4x4_x5_375_split.xclbin</t>
+        </is>
+      </c>
+      <c r="P10" s="2" t="n">
+        <v>329</v>
+      </c>
+      <c r="Q10" s="2" t="inlineStr">
+        <is>
+          <t>60 s power soak, host calculation counts x MACs per calculation; static = idle after the soak, dynamic = load - idle</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>5 tenants</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="n">
+        <v>0.7123</v>
+      </c>
+      <c r="D11" s="2" t="n">
+        <v>0.1784</v>
+      </c>
+      <c r="E11" s="2" t="n">
+        <v>0.8907</v>
+      </c>
+      <c r="F11" s="2" t="n">
+        <v>47.209</v>
+      </c>
+      <c r="G11" s="2" t="n">
+        <v>42.047</v>
+      </c>
+      <c r="H11" s="2" t="n">
+        <v>33.626</v>
+      </c>
+      <c r="I11" s="2" t="n">
+        <v>8.420999999999999</v>
+      </c>
+      <c r="J11" s="2" t="n">
+        <v>10.252</v>
+      </c>
+      <c r="K11" s="2" t="n">
+        <v>8.526999999999999</v>
+      </c>
+      <c r="L11" s="2" t="n">
+        <v>79.97</v>
+      </c>
+      <c r="M11" s="2" t="inlineStr">
+        <is>
+          <t>All 2:32</t>
+        </is>
+      </c>
+      <c r="N11" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="O11" s="2" t="inlineStr">
+        <is>
+          <t>sparse_4x4_x5_375_split.xclbin</t>
+        </is>
+      </c>
+      <c r="P11" s="2" t="n">
+        <v>329</v>
+      </c>
+      <c r="Q11" s="2" t="inlineStr">
+        <is>
+          <t>60 s power soak, host calculation counts x MACs per calculation; static = idle after the soak, dynamic = load - idle</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:Q11"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="29" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="30" customWidth="1" min="6" max="6"/>
+    <col width="30" customWidth="1" min="7" max="7"/>
+    <col width="30" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>metric</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>ratio_scaleout_over_scaleup</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>scaleout_value</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>scaleup_value</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>unit</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>scaleout</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>scaleup</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>basis</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>HBM channels</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C2" s="2" t="n">
+        <v>24</v>
+      </c>
+      <c r="D2" s="2" t="n">
+        <v>24</v>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>channels</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>4 x 4x4 tenants, sparse_4x4_x4_375.xclbin</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>one 4x24 engine, family build</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>the controlled variable: the same channel budget</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Kernel clock</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="n">
+        <v>1.2467</v>
+      </c>
+      <c r="C3" s="2" t="n">
+        <v>374</v>
+      </c>
+      <c r="D3" s="2" t="n">
+        <v>300</v>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>MHz</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>4 x 4x4 tenants, sparse_4x4_x4_375.xclbin</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>one 4x24 engine, family build</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>runtime clock of each bitstream</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>MACs per cycle</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="n">
+        <v>0.6667</v>
+      </c>
+      <c r="C4" s="2" t="n">
+        <v>128</v>
+      </c>
+      <c r="D4" s="2" t="n">
+        <v>192</v>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>MACs/cycle</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>4 x 4x4 tenants, sparse_4x4_x4_375.xclbin</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>one 4x24 engine, family build</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>4 x 32 vs 96 blocks x 2 (DSPs 512 vs 768)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Throughput</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="n">
+        <v>0.8307</v>
+      </c>
+      <c r="C5" s="2" t="n">
+        <v>47.37</v>
+      </c>
+      <c r="D5" s="2" t="n">
+        <v>57.025</v>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>GMAC/s</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>4 x 4x4 tenants, sparse_4x4_x4_375.xclbin</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>one 4x24 engine, family build</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>steady state: x4 = MACs / (active span - 189 us fixed cost), all four tenants running; 4x24 = ss_gflops_act_MIXED / 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Board power</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="n">
+        <v>0.9979</v>
+      </c>
+      <c r="C6" s="2" t="n">
+        <v>40.345</v>
+      </c>
+      <c r="D6" s="2" t="n">
+        <v>40.43</v>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>4 x 4x4 tenants, sparse_4x4_x4_375.xclbin</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>one 4x24 engine, family build</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>60 s MIXED soak, board load</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Energy per MAC</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="n">
+        <v>1.2013</v>
+      </c>
+      <c r="C7" s="2" t="n">
+        <v>0.8517</v>
+      </c>
+      <c r="D7" s="2" t="n">
+        <v>0.709</v>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>nJ/MAC</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>4 x 4x4 tenants, sparse_4x4_x4_375.xclbin</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>one 4x24 engine, family build</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>soak board power / steady-state GMAC/s (the family's per-W method)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:H7"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:K14"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="11" customWidth="1" min="8" max="8"/>
+    <col width="20" customWidth="1" min="9" max="9"/>
+    <col width="10" customWidth="1" min="10" max="10"/>
+    <col width="30" customWidth="1" min="11" max="11"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>build_label</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>idle_vccint_W</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>idle_rest_W</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>idle_board_W</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>hbm_channels</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>build</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>kind</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>clock_mhz</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>uses_channel_16_up</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>n_soaks</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>4x4 (6 ch)</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="n">
+        <v>6.048</v>
+      </c>
+      <c r="C2" s="2" t="n">
+        <v>19.395</v>
+      </c>
+      <c r="D2" s="2" t="n">
+        <v>25.443</v>
+      </c>
+      <c r="E2" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>4x4</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>single engine</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="n">
+        <v>400</v>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>results/family_measurements/4x4/power_4x4_400MHz.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>8x4 (10 ch)</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="n">
+        <v>6.56</v>
+      </c>
+      <c r="C3" s="2" t="n">
+        <v>20.091</v>
+      </c>
+      <c r="D3" s="2" t="n">
+        <v>26.651</v>
+      </c>
+      <c r="E3" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>8x4</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>single engine</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="n">
+        <v>375</v>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>results/family_measurements/8x4/power_8x4_375MHz.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>2 x 4x4 (12 ch)</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="n">
+        <v>6.655</v>
+      </c>
+      <c r="C4" s="2" t="n">
+        <v>20.108</v>
+      </c>
+      <c r="D4" s="2" t="n">
+        <v>26.764</v>
+      </c>
+      <c r="E4" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>4x4_x2</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>multi-tenant</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="n">
+        <v>394</v>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="K4" s="2" t="inlineStr">
+        <is>
+          <t>multi_x2_394MHz.csv, multi_x2_394MHz_all2to32.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>16x3 (13 ch)</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="n">
+        <v>7.139</v>
+      </c>
+      <c r="C5" s="2" t="n">
+        <v>20.448</v>
+      </c>
+      <c r="D5" s="2" t="n">
+        <v>27.587</v>
+      </c>
+      <c r="E5" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>16x3</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>single engine</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="n">
+        <v>350</v>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J5" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="K5" s="2" t="inlineStr">
+        <is>
+          <t>results/family_measurements/16x3/power_16x3_350MHz.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>8x8 (17 ch)</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="n">
+        <v>7.528</v>
+      </c>
+      <c r="C6" s="2" t="n">
+        <v>23.309</v>
+      </c>
+      <c r="D6" s="2" t="n">
+        <v>30.837</v>
+      </c>
+      <c r="E6" s="2" t="n">
+        <v>17</v>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>8x8</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>single engine</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="n">
+        <v>325</v>
+      </c>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="J6" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="K6" s="2" t="inlineStr">
+        <is>
+          <t>results/family_measurements/8x8/power_8x8_325MHz.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>3 x 4x4 (18 ch)</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="n">
+        <v>7.514</v>
+      </c>
+      <c r="C7" s="2" t="n">
+        <v>23.353</v>
+      </c>
+      <c r="D7" s="2" t="n">
+        <v>30.867</v>
+      </c>
+      <c r="E7" s="2" t="n">
+        <v>18</v>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>4x4_x3</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>multi-tenant</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="n">
+        <v>399</v>
+      </c>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="J7" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="K7" s="2" t="inlineStr">
+        <is>
+          <t>multi_x3_399MHz.csv, multi_x3_399MHz_all2to32.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>2 x 8x4 (20 ch)</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="n">
+        <v>7.716</v>
+      </c>
+      <c r="C8" s="2" t="n">
+        <v>23.669</v>
+      </c>
+      <c r="D8" s="2" t="n">
+        <v>31.386</v>
+      </c>
+      <c r="E8" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>8x4_x2</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>multi-tenant</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="n">
+        <v>361</v>
+      </c>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="J8" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="K8" s="2" t="inlineStr">
+        <is>
+          <t>multi_8x4_x2_361MHz.csv, multi_8x4_x2_361MHz_all2to32.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>4x24 (24 ch)</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="n">
+        <v>8.287000000000001</v>
+      </c>
+      <c r="C9" s="2" t="n">
+        <v>24.259</v>
+      </c>
+      <c r="D9" s="2" t="n">
+        <v>32.546</v>
+      </c>
+      <c r="E9" s="2" t="n">
+        <v>24</v>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>4x24</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>single engine</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="n">
+        <v>300</v>
+      </c>
+      <c r="I9" s="2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="J9" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="K9" s="2" t="inlineStr">
+        <is>
+          <t>results/family_measurements/4x24/power_4x24_300MHz.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>4 x 4x4 (24 ch)</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="n">
+        <v>8.365</v>
+      </c>
+      <c r="C10" s="2" t="n">
+        <v>24.416</v>
+      </c>
+      <c r="D10" s="2" t="n">
+        <v>32.782</v>
+      </c>
+      <c r="E10" s="2" t="n">
+        <v>24</v>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>4x4_x4</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>multi-tenant</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="n">
+        <v>374</v>
+      </c>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="J10" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="K10" s="2" t="inlineStr">
+        <is>
+          <t>multi_x4_374MHz.csv, multi_x4_374MHz_all2to32.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>2 x 16x3 (26 ch)</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="n">
+        <v>9.048</v>
+      </c>
+      <c r="C11" s="2" t="n">
+        <v>25.084</v>
+      </c>
+      <c r="D11" s="2" t="n">
+        <v>34.132</v>
+      </c>
+      <c r="E11" s="2" t="n">
+        <v>26</v>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>16x3_x2</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>multi-tenant</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="n">
+        <v>341</v>
+      </c>
+      <c r="I11" s="2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="J11" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="K11" s="2" t="inlineStr">
+        <is>
+          <t>multi_16x3_x2_341MHz.csv, multi_16x3_x2_341MHz_all2to32.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>5 x 4x4 (30 ch)</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="n">
+        <v>8.640000000000001</v>
+      </c>
+      <c r="C12" s="2" t="n">
+        <v>25.025</v>
+      </c>
+      <c r="D12" s="2" t="n">
+        <v>33.665</v>
+      </c>
+      <c r="E12" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>4x4_x5</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>multi-tenant</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="n">
+        <v>329</v>
+      </c>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="J12" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="K12" s="2" t="inlineStr">
+        <is>
+          <t>multi_x5_329MHz.csv, multi_x5_329MHz_all2to32.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>3 x 8x4 (30 ch)</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="n">
+        <v>8.877000000000001</v>
+      </c>
+      <c r="C13" s="2" t="n">
+        <v>25.183</v>
+      </c>
+      <c r="D13" s="2" t="n">
+        <v>34.061</v>
+      </c>
+      <c r="E13" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>8x4_x3</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>multi-tenant</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="n">
+        <v>354</v>
+      </c>
+      <c r="I13" s="2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="J13" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="K13" s="2" t="inlineStr">
+        <is>
+          <t>multi_8x4_x3_354MHz.csv, multi_8x4_x3_354MHz_all2to32.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>4x32 (32 ch)</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="n">
+        <v>8.612</v>
+      </c>
+      <c r="C14" s="2" t="n">
+        <v>25.039</v>
+      </c>
+      <c r="D14" s="2" t="n">
+        <v>33.651</v>
+      </c>
+      <c r="E14" s="2" t="n">
+        <v>32</v>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>4x32</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>single engine</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="n">
+        <v>250</v>
+      </c>
+      <c r="I14" s="2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="J14" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="K14" s="2" t="inlineStr">
+        <is>
+          <t>results/family_measurements/4x32/power_4x32_250MHz.csv</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:K14"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:AC14"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="26" customWidth="1" min="4" max="4"/>
+    <col width="27" customWidth="1" min="5" max="5"/>
+    <col width="25" customWidth="1" min="6" max="6"/>
+    <col width="26" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
+    <col width="17" customWidth="1" min="9" max="9"/>
+    <col width="27" customWidth="1" min="10" max="10"/>
+    <col width="26" customWidth="1" min="11" max="11"/>
+    <col width="15" customWidth="1" min="12" max="12"/>
+    <col width="18" customWidth="1" min="13" max="13"/>
+    <col width="14" customWidth="1" min="14" max="14"/>
+    <col width="10" customWidth="1" min="15" max="15"/>
+    <col width="14" customWidth="1" min="16" max="16"/>
+    <col width="13" customWidth="1" min="17" max="17"/>
+    <col width="16" customWidth="1" min="18" max="18"/>
+    <col width="11" customWidth="1" min="19" max="19"/>
+    <col width="10" customWidth="1" min="20" max="20"/>
+    <col width="13" customWidth="1" min="21" max="21"/>
+    <col width="20" customWidth="1" min="22" max="22"/>
+    <col width="25" customWidth="1" min="23" max="23"/>
+    <col width="14" customWidth="1" min="24" max="24"/>
+    <col width="14" customWidth="1" min="25" max="25"/>
+    <col width="11" customWidth="1" min="26" max="26"/>
+    <col width="10" customWidth="1" min="27" max="27"/>
+    <col width="30" customWidth="1" min="28" max="28"/>
+    <col width="30" customWidth="1" min="29" max="29"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>config_label</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>gmac_s_single</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>gmac_s_multi</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>static_nJ_per_MAC_single</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>dynamic_nJ_per_MAC_single</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>static_nJ_per_MAC_multi</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>dynamic_nJ_per_MAC_multi</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>clock_mhz_single</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>clock_mhz_multi</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>gmac_s_per_channel_single</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>gmac_s_per_channel_multi</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>kind</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>configuration</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>engine_shape</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>tenants</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>hbm_channels</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>lanes_total</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>macs_per_cycle</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>clock_mhz</t>
+        </is>
+      </c>
+      <c r="T1" s="1" t="inlineStr">
+        <is>
+          <t>gmac_s</t>
+        </is>
+      </c>
+      <c r="U1" s="1" t="inlineStr">
+        <is>
+          <t>pct_of_peak</t>
+        </is>
+      </c>
+      <c r="V1" s="1" t="inlineStr">
+        <is>
+          <t>gmac_s_per_channel</t>
+        </is>
+      </c>
+      <c r="W1" s="1" t="inlineStr">
+        <is>
+          <t>energy_total_nJ_per_MAC</t>
+        </is>
+      </c>
+      <c r="X1" s="1" t="inlineStr">
+        <is>
+          <t>board_load_W</t>
+        </is>
+      </c>
+      <c r="Y1" s="1" t="inlineStr">
+        <is>
+          <t>board_idle_W</t>
+        </is>
+      </c>
+      <c r="Z1" s="1" t="inlineStr">
+        <is>
+          <t>floorplan</t>
+        </is>
+      </c>
+      <c r="AA1" s="1" t="inlineStr">
+        <is>
+          <t>status</t>
+        </is>
+      </c>
+      <c r="AB1" s="1" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+      <c r="AC1" s="1" t="inlineStr">
+        <is>
+          <t>estimator</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>4x4 (6 ch)</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="n">
+        <v>12.615</v>
+      </c>
+      <c r="D2" s="2" t="n">
+        <v>1.9997</v>
+      </c>
+      <c r="E2" s="2" t="n">
+        <v>0.1669</v>
+      </c>
+      <c r="H2" s="2" t="n">
+        <v>400</v>
+      </c>
+      <c r="J2" s="2" t="n">
+        <v>2.1025</v>
+      </c>
+      <c r="L2" s="2" t="inlineStr">
+        <is>
+          <t>single engine</t>
+        </is>
+      </c>
+      <c r="M2" s="2" t="inlineStr">
+        <is>
+          <t>one 4x4 engine</t>
+        </is>
+      </c>
+      <c r="N2" s="2" t="inlineStr">
+        <is>
+          <t>4x4</t>
+        </is>
+      </c>
+      <c r="O2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="P2" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="Q2" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="R2" s="2" t="n">
+        <v>32</v>
+      </c>
+      <c r="S2" s="2" t="n">
+        <v>400</v>
+      </c>
+      <c r="T2" s="2" t="n">
+        <v>12.615</v>
+      </c>
+      <c r="U2" s="2" t="n">
+        <v>98.55</v>
+      </c>
+      <c r="V2" s="2" t="n">
+        <v>2.1025</v>
+      </c>
+      <c r="W2" s="2" t="n">
+        <v>2.1666</v>
+      </c>
+      <c r="X2" s="2" t="n">
+        <v>27.332</v>
+      </c>
+      <c r="Y2" s="2" t="n">
+        <v>25.226</v>
+      </c>
+      <c r="Z2" s="2" t="inlineStr">
+        <is>
+          <t>SLR0</t>
+        </is>
+      </c>
+      <c r="AA2" s="2" t="inlineStr">
+        <is>
+          <t>measured</t>
+        </is>
+      </c>
+      <c r="AB2" s="2" t="inlineStr">
+        <is>
+          <t>GEMV_Family_Measured.csv, family_measurements/4x4/power_4x4_400MHz.csv</t>
+        </is>
+      </c>
+      <c r="AC2" s="2" t="inlineStr">
+        <is>
+          <t>steady state: ss_gflops_act_MIXED / 2; energy = MIXED soak power / that</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>8x4 (10 ch)</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="n">
+        <v>23.715</v>
+      </c>
+      <c r="D3" s="2" t="n">
+        <v>1.1236</v>
+      </c>
+      <c r="E3" s="2" t="n">
+        <v>0.1325</v>
+      </c>
+      <c r="H3" s="2" t="n">
+        <v>375</v>
+      </c>
+      <c r="J3" s="2" t="n">
+        <v>2.3715</v>
+      </c>
+      <c r="L3" s="2" t="inlineStr">
+        <is>
+          <t>single engine</t>
+        </is>
+      </c>
+      <c r="M3" s="2" t="inlineStr">
+        <is>
+          <t>one 8x4 engine</t>
+        </is>
+      </c>
+      <c r="N3" s="2" t="inlineStr">
+        <is>
+          <t>8x4</t>
+        </is>
+      </c>
+      <c r="O3" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="P3" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q3" s="2" t="n">
+        <v>32</v>
+      </c>
+      <c r="R3" s="2" t="n">
+        <v>64</v>
+      </c>
+      <c r="S3" s="2" t="n">
+        <v>375</v>
+      </c>
+      <c r="T3" s="2" t="n">
+        <v>23.715</v>
+      </c>
+      <c r="U3" s="2" t="n">
+        <v>98.81</v>
+      </c>
+      <c r="V3" s="2" t="n">
+        <v>2.3715</v>
+      </c>
+      <c r="W3" s="2" t="n">
+        <v>1.2562</v>
+      </c>
+      <c r="X3" s="2" t="n">
+        <v>29.79</v>
+      </c>
+      <c r="Y3" s="2" t="n">
+        <v>26.647</v>
+      </c>
+      <c r="Z3" s="2" t="inlineStr">
+        <is>
+          <t>SLR0</t>
+        </is>
+      </c>
+      <c r="AA3" s="2" t="inlineStr">
+        <is>
+          <t>measured</t>
+        </is>
+      </c>
+      <c r="AB3" s="2" t="inlineStr">
+        <is>
+          <t>GEMV_Family_Measured.csv, family_measurements/8x4/power_8x4_375MHz.csv</t>
+        </is>
+      </c>
+      <c r="AC3" s="2" t="inlineStr">
+        <is>
+          <t>steady state: ss_gflops_act_MIXED / 2; energy = MIXED soak power / that</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>2 x 4x4 (12 ch)</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="n">
+        <v>24.997</v>
+      </c>
+      <c r="F4" s="2" t="n">
+        <v>1.0717</v>
+      </c>
+      <c r="G4" s="2" t="n">
+        <v>0.1582</v>
+      </c>
+      <c r="I4" s="2" t="n">
+        <v>394</v>
+      </c>
+      <c r="K4" s="2" t="n">
+        <v>2.0831</v>
+      </c>
+      <c r="L4" s="2" t="inlineStr">
+        <is>
+          <t>multi-tenant</t>
+        </is>
+      </c>
+      <c r="M4" s="2" t="inlineStr">
+        <is>
+          <t>2 x 4x4 tenants</t>
+        </is>
+      </c>
+      <c r="N4" s="2" t="inlineStr">
+        <is>
+          <t>4x4</t>
+        </is>
+      </c>
+      <c r="O4" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="P4" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="Q4" s="2" t="n">
+        <v>32</v>
+      </c>
+      <c r="R4" s="2" t="n">
+        <v>64</v>
+      </c>
+      <c r="S4" s="2" t="n">
+        <v>394</v>
+      </c>
+      <c r="T4" s="2" t="n">
+        <v>24.997</v>
+      </c>
+      <c r="U4" s="2" t="n">
+        <v>99.13</v>
+      </c>
+      <c r="V4" s="2" t="n">
+        <v>2.0831</v>
+      </c>
+      <c r="W4" s="2" t="n">
+        <v>1.2299</v>
+      </c>
+      <c r="X4" s="2" t="n">
+        <v>30.744</v>
+      </c>
+      <c r="Y4" s="2" t="n">
+        <v>26.789</v>
+      </c>
+      <c r="Z4" s="2" t="inlineStr">
+        <is>
+          <t>SLR0</t>
+        </is>
+      </c>
+      <c r="AA4" s="2" t="inlineStr">
+        <is>
+          <t>measured</t>
+        </is>
+      </c>
+      <c r="AB4" s="2" t="inlineStr">
+        <is>
+          <t>multi_x2_394MHz.csv (sparse_4x4_x2_400.xclbin)</t>
+        </is>
+      </c>
+      <c r="AC4" s="2" t="inlineStr">
+        <is>
+          <t>steady state: sum over tenants of MACs / (active span - a), all tenants running; energy = full-set MIXED soak power / that</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>16x3 (13 ch)</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="n">
+        <v>33.1</v>
+      </c>
+      <c r="D5" s="2" t="n">
+        <v>0.8308</v>
+      </c>
+      <c r="E5" s="2" t="n">
+        <v>0.143</v>
+      </c>
+      <c r="H5" s="2" t="n">
+        <v>350</v>
+      </c>
+      <c r="J5" s="2" t="n">
+        <v>2.5462</v>
+      </c>
+      <c r="L5" s="2" t="inlineStr">
+        <is>
+          <t>single engine</t>
+        </is>
+      </c>
+      <c r="M5" s="2" t="inlineStr">
+        <is>
+          <t>one 16x3 engine</t>
+        </is>
+      </c>
+      <c r="N5" s="2" t="inlineStr">
+        <is>
+          <t>16x3</t>
+        </is>
+      </c>
+      <c r="O5" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="P5" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="Q5" s="2" t="n">
+        <v>48</v>
+      </c>
+      <c r="R5" s="2" t="n">
+        <v>96</v>
+      </c>
+      <c r="S5" s="2" t="n">
+        <v>350</v>
+      </c>
+      <c r="T5" s="2" t="n">
+        <v>33.1</v>
+      </c>
+      <c r="U5" s="2" t="n">
+        <v>98.51000000000001</v>
+      </c>
+      <c r="V5" s="2" t="n">
+        <v>2.5462</v>
+      </c>
+      <c r="W5" s="2" t="n">
+        <v>0.9739</v>
+      </c>
+      <c r="X5" s="2" t="n">
+        <v>32.235</v>
+      </c>
+      <c r="Y5" s="2" t="n">
+        <v>27.501</v>
+      </c>
+      <c r="Z5" s="2" t="inlineStr">
+        <is>
+          <t>SLR0</t>
+        </is>
+      </c>
+      <c r="AA5" s="2" t="inlineStr">
+        <is>
+          <t>measured</t>
+        </is>
+      </c>
+      <c r="AB5" s="2" t="inlineStr">
+        <is>
+          <t>GEMV_Family_Measured.csv, family_measurements/16x3/power_16x3_350MHz.csv</t>
+        </is>
+      </c>
+      <c r="AC5" s="2" t="inlineStr">
+        <is>
+          <t>steady state: ss_gflops_act_MIXED / 2; energy = MIXED soak power / that</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>8x8 (17 ch)</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="n">
+        <v>41.125</v>
+      </c>
+      <c r="D6" s="2" t="n">
+        <v>0.751</v>
+      </c>
+      <c r="E6" s="2" t="n">
+        <v>0.1314</v>
+      </c>
+      <c r="H6" s="2" t="n">
+        <v>325</v>
+      </c>
+      <c r="J6" s="2" t="n">
+        <v>2.4191</v>
+      </c>
+      <c r="L6" s="2" t="inlineStr">
+        <is>
+          <t>single engine</t>
+        </is>
+      </c>
+      <c r="M6" s="2" t="inlineStr">
+        <is>
+          <t>one 8x8 engine</t>
+        </is>
+      </c>
+      <c r="N6" s="2" t="inlineStr">
+        <is>
+          <t>8x8</t>
+        </is>
+      </c>
+      <c r="O6" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="P6" s="2" t="n">
+        <v>17</v>
+      </c>
+      <c r="Q6" s="2" t="n">
+        <v>64</v>
+      </c>
+      <c r="R6" s="2" t="n">
+        <v>128</v>
+      </c>
+      <c r="S6" s="2" t="n">
+        <v>325</v>
+      </c>
+      <c r="T6" s="2" t="n">
+        <v>41.125</v>
+      </c>
+      <c r="U6" s="2" t="n">
+        <v>98.86</v>
+      </c>
+      <c r="V6" s="2" t="n">
+        <v>2.4191</v>
+      </c>
+      <c r="W6" s="2" t="n">
+        <v>0.8823</v>
+      </c>
+      <c r="X6" s="2" t="n">
+        <v>36.286</v>
+      </c>
+      <c r="Y6" s="2" t="n">
+        <v>30.883</v>
+      </c>
+      <c r="Z6" s="2" t="inlineStr">
+        <is>
+          <t>split</t>
+        </is>
+      </c>
+      <c r="AA6" s="2" t="inlineStr">
+        <is>
+          <t>measured</t>
+        </is>
+      </c>
+      <c r="AB6" s="2" t="inlineStr">
+        <is>
+          <t>GEMV_Family_Measured.csv, family_measurements/8x8/power_8x8_325MHz.csv</t>
+        </is>
+      </c>
+      <c r="AC6" s="2" t="inlineStr">
+        <is>
+          <t>steady state: ss_gflops_act_MIXED / 2; energy = MIXED soak power / that</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>3 x 4x4 (18 ch)</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="n">
+        <v>37.915</v>
+      </c>
+      <c r="F7" s="2" t="n">
+        <v>0.8166</v>
+      </c>
+      <c r="G7" s="2" t="n">
+        <v>0.164</v>
+      </c>
+      <c r="I7" s="2" t="n">
+        <v>399</v>
+      </c>
+      <c r="K7" s="2" t="n">
+        <v>2.1064</v>
+      </c>
+      <c r="L7" s="2" t="inlineStr">
+        <is>
+          <t>multi-tenant</t>
+        </is>
+      </c>
+      <c r="M7" s="2" t="inlineStr">
+        <is>
+          <t>3 x 4x4 tenants</t>
+        </is>
+      </c>
+      <c r="N7" s="2" t="inlineStr">
+        <is>
+          <t>4x4</t>
+        </is>
+      </c>
+      <c r="O7" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="P7" s="2" t="n">
+        <v>18</v>
+      </c>
+      <c r="Q7" s="2" t="n">
+        <v>48</v>
+      </c>
+      <c r="R7" s="2" t="n">
+        <v>96</v>
+      </c>
+      <c r="S7" s="2" t="n">
+        <v>399</v>
+      </c>
+      <c r="T7" s="2" t="n">
+        <v>37.915</v>
+      </c>
+      <c r="U7" s="2" t="n">
+        <v>98.98999999999999</v>
+      </c>
+      <c r="V7" s="2" t="n">
+        <v>2.1064</v>
+      </c>
+      <c r="W7" s="2" t="n">
+        <v>0.9806</v>
+      </c>
+      <c r="X7" s="2" t="n">
+        <v>37.179</v>
+      </c>
+      <c r="Y7" s="2" t="n">
+        <v>30.96</v>
+      </c>
+      <c r="Z7" s="2" t="inlineStr">
+        <is>
+          <t>SLR0</t>
+        </is>
+      </c>
+      <c r="AA7" s="2" t="inlineStr">
+        <is>
+          <t>measured</t>
+        </is>
+      </c>
+      <c r="AB7" s="2" t="inlineStr">
+        <is>
+          <t>multi_x3_399MHz.csv (sparse_4x4_x3_400.xclbin)</t>
+        </is>
+      </c>
+      <c r="AC7" s="2" t="inlineStr">
+        <is>
+          <t>steady state: sum over tenants of MACs / (active span - a), all tenants running; energy = full-set MIXED soak power / that</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>2 x 8x4 (20 ch)</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="n">
+        <v>45.591</v>
+      </c>
+      <c r="F8" s="2" t="n">
+        <v>0.6896</v>
+      </c>
+      <c r="G8" s="2" t="n">
+        <v>0.149</v>
+      </c>
+      <c r="I8" s="2" t="n">
+        <v>361</v>
+      </c>
+      <c r="K8" s="2" t="n">
+        <v>2.2795</v>
+      </c>
+      <c r="L8" s="2" t="inlineStr">
+        <is>
+          <t>multi-tenant</t>
+        </is>
+      </c>
+      <c r="M8" s="2" t="inlineStr">
+        <is>
+          <t>2 x 8x4 tenants</t>
+        </is>
+      </c>
+      <c r="N8" s="2" t="inlineStr">
+        <is>
+          <t>8x4</t>
+        </is>
+      </c>
+      <c r="O8" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="P8" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="Q8" s="2" t="n">
+        <v>64</v>
+      </c>
+      <c r="R8" s="2" t="n">
+        <v>128</v>
+      </c>
+      <c r="S8" s="2" t="n">
+        <v>361</v>
+      </c>
+      <c r="T8" s="2" t="n">
+        <v>45.591</v>
+      </c>
+      <c r="U8" s="2" t="n">
+        <v>98.66</v>
+      </c>
+      <c r="V8" s="2" t="n">
+        <v>2.2795</v>
+      </c>
+      <c r="W8" s="2" t="n">
+        <v>0.8386</v>
+      </c>
+      <c r="X8" s="2" t="n">
+        <v>38.233</v>
+      </c>
+      <c r="Y8" s="2" t="n">
+        <v>31.438</v>
+      </c>
+      <c r="Z8" s="2" t="inlineStr">
+        <is>
+          <t>SLR0</t>
+        </is>
+      </c>
+      <c r="AA8" s="2" t="inlineStr">
+        <is>
+          <t>measured</t>
+        </is>
+      </c>
+      <c r="AB8" s="2" t="inlineStr">
+        <is>
+          <t>multi_8x4_x2_361MHz.csv (sparse_8x4_x2_375.xclbin)</t>
+        </is>
+      </c>
+      <c r="AC8" s="2" t="inlineStr">
+        <is>
+          <t>steady state: sum over tenants of MACs / (active span - a), all tenants running; energy = full-set MIXED soak power / that</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>4x24 (24 ch)</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="n">
+        <v>57.025</v>
+      </c>
+      <c r="D9" s="2" t="n">
+        <v>0.5723</v>
+      </c>
+      <c r="E9" s="2" t="n">
+        <v>0.1367</v>
+      </c>
+      <c r="H9" s="2" t="n">
+        <v>300</v>
+      </c>
+      <c r="J9" s="2" t="n">
+        <v>2.376</v>
+      </c>
+      <c r="L9" s="2" t="inlineStr">
+        <is>
+          <t>single engine</t>
+        </is>
+      </c>
+      <c r="M9" s="2" t="inlineStr">
+        <is>
+          <t>one 4x24 engine</t>
+        </is>
+      </c>
+      <c r="N9" s="2" t="inlineStr">
+        <is>
+          <t>4x24</t>
+        </is>
+      </c>
+      <c r="O9" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="P9" s="2" t="n">
+        <v>24</v>
+      </c>
+      <c r="Q9" s="2" t="n">
+        <v>96</v>
+      </c>
+      <c r="R9" s="2" t="n">
+        <v>192</v>
+      </c>
+      <c r="S9" s="2" t="n">
+        <v>300</v>
+      </c>
+      <c r="T9" s="2" t="n">
+        <v>57.025</v>
+      </c>
+      <c r="U9" s="2" t="n">
+        <v>99</v>
+      </c>
+      <c r="V9" s="2" t="n">
+        <v>2.376</v>
+      </c>
+      <c r="W9" s="2" t="n">
+        <v>0.709</v>
+      </c>
+      <c r="X9" s="2" t="n">
+        <v>40.43</v>
+      </c>
+      <c r="Y9" s="2" t="n">
+        <v>32.633</v>
+      </c>
+      <c r="Z9" s="2" t="inlineStr">
+        <is>
+          <t>split</t>
+        </is>
+      </c>
+      <c r="AA9" s="2" t="inlineStr">
+        <is>
+          <t>measured</t>
+        </is>
+      </c>
+      <c r="AB9" s="2" t="inlineStr">
+        <is>
+          <t>GEMV_Family_Measured.csv, family_measurements/4x24/power_4x24_300MHz.csv</t>
+        </is>
+      </c>
+      <c r="AC9" s="2" t="inlineStr">
+        <is>
+          <t>steady state: ss_gflops_act_MIXED / 2; energy = MIXED soak power / that</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>4 x 4x4 (24 ch)</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="n">
+        <v>47.37</v>
+      </c>
+      <c r="F10" s="2" t="n">
+        <v>0.6975</v>
+      </c>
+      <c r="G10" s="2" t="n">
+        <v>0.1542</v>
+      </c>
+      <c r="I10" s="2" t="n">
+        <v>374</v>
+      </c>
+      <c r="K10" s="2" t="n">
+        <v>1.9738</v>
+      </c>
+      <c r="L10" s="2" t="inlineStr">
+        <is>
+          <t>multi-tenant</t>
+        </is>
+      </c>
+      <c r="M10" s="2" t="inlineStr">
+        <is>
+          <t>4 x 4x4 tenants</t>
+        </is>
+      </c>
+      <c r="N10" s="2" t="inlineStr">
+        <is>
+          <t>4x4</t>
+        </is>
+      </c>
+      <c r="O10" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="P10" s="2" t="n">
+        <v>24</v>
+      </c>
+      <c r="Q10" s="2" t="n">
+        <v>64</v>
+      </c>
+      <c r="R10" s="2" t="n">
+        <v>128</v>
+      </c>
+      <c r="S10" s="2" t="n">
+        <v>374</v>
+      </c>
+      <c r="T10" s="2" t="n">
+        <v>47.37</v>
+      </c>
+      <c r="U10" s="2" t="n">
+        <v>98.95</v>
+      </c>
+      <c r="V10" s="2" t="n">
+        <v>1.9738</v>
+      </c>
+      <c r="W10" s="2" t="n">
+        <v>0.8517</v>
+      </c>
+      <c r="X10" s="2" t="n">
+        <v>40.345</v>
+      </c>
+      <c r="Y10" s="2" t="n">
+        <v>33.041</v>
+      </c>
+      <c r="Z10" s="2" t="inlineStr">
+        <is>
+          <t>SLR0</t>
+        </is>
+      </c>
+      <c r="AA10" s="2" t="inlineStr">
+        <is>
+          <t>measured</t>
+        </is>
+      </c>
+      <c r="AB10" s="2" t="inlineStr">
+        <is>
+          <t>multi_x4_374MHz.csv (sparse_4x4_x4_375.xclbin)</t>
+        </is>
+      </c>
+      <c r="AC10" s="2" t="inlineStr">
+        <is>
+          <t>steady state: sum over tenants of MACs / (active span - a), all tenants running; energy = full-set MIXED soak power / that</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>2 x 16x3 (26 ch)</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="n">
+        <v>64.642</v>
+      </c>
+      <c r="F11" s="2" t="n">
+        <v>0.5318000000000001</v>
+      </c>
+      <c r="G11" s="2" t="n">
+        <v>0.1252</v>
+      </c>
+      <c r="I11" s="2" t="n">
+        <v>341</v>
+      </c>
+      <c r="K11" s="2" t="n">
+        <v>2.4862</v>
+      </c>
+      <c r="L11" s="2" t="inlineStr">
+        <is>
+          <t>multi-tenant</t>
+        </is>
+      </c>
+      <c r="M11" s="2" t="inlineStr">
+        <is>
+          <t>2 x 16x3 tenants</t>
+        </is>
+      </c>
+      <c r="N11" s="2" t="inlineStr">
+        <is>
+          <t>16x3</t>
+        </is>
+      </c>
+      <c r="O11" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="P11" s="2" t="n">
+        <v>26</v>
+      </c>
+      <c r="Q11" s="2" t="n">
+        <v>96</v>
+      </c>
+      <c r="R11" s="2" t="n">
+        <v>192</v>
+      </c>
+      <c r="S11" s="2" t="n">
+        <v>341</v>
+      </c>
+      <c r="T11" s="2" t="n">
+        <v>64.642</v>
+      </c>
+      <c r="U11" s="2" t="n">
+        <v>98.73</v>
+      </c>
+      <c r="V11" s="2" t="n">
+        <v>2.4862</v>
+      </c>
+      <c r="W11" s="2" t="n">
+        <v>0.657</v>
+      </c>
+      <c r="X11" s="2" t="n">
+        <v>42.468</v>
+      </c>
+      <c r="Y11" s="2" t="n">
+        <v>34.378</v>
+      </c>
+      <c r="Z11" s="2" t="inlineStr">
+        <is>
+          <t>split</t>
+        </is>
+      </c>
+      <c r="AA11" s="2" t="inlineStr">
+        <is>
+          <t>measured</t>
+        </is>
+      </c>
+      <c r="AB11" s="2" t="inlineStr">
+        <is>
+          <t>multi_16x3_x2_341MHz.csv (sparse_16x3_x2_375.xclbin)</t>
+        </is>
+      </c>
+      <c r="AC11" s="2" t="inlineStr">
+        <is>
+          <t>steady state: sum over tenants of MACs / (active span - a), all tenants running; energy = full-set MIXED soak power / that</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>5 x 4x4 (30 ch)</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="n">
+        <v>51.718</v>
+      </c>
+      <c r="F12" s="2" t="n">
+        <v>0.6529</v>
+      </c>
+      <c r="G12" s="2" t="n">
+        <v>0.1628</v>
+      </c>
+      <c r="I12" s="2" t="n">
+        <v>329</v>
+      </c>
+      <c r="K12" s="2" t="n">
+        <v>1.7239</v>
+      </c>
+      <c r="L12" s="2" t="inlineStr">
+        <is>
+          <t>multi-tenant</t>
+        </is>
+      </c>
+      <c r="M12" s="2" t="inlineStr">
+        <is>
+          <t>5 x 4x4 tenants</t>
+        </is>
+      </c>
+      <c r="N12" s="2" t="inlineStr">
+        <is>
+          <t>4x4</t>
+        </is>
+      </c>
+      <c r="O12" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="P12" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="Q12" s="2" t="n">
+        <v>80</v>
+      </c>
+      <c r="R12" s="2" t="n">
+        <v>160</v>
+      </c>
+      <c r="S12" s="2" t="n">
+        <v>329</v>
+      </c>
+      <c r="T12" s="2" t="n">
+        <v>51.718</v>
+      </c>
+      <c r="U12" s="2" t="n">
+        <v>98.25</v>
+      </c>
+      <c r="V12" s="2" t="n">
+        <v>1.7239</v>
+      </c>
+      <c r="W12" s="2" t="n">
+        <v>0.8157</v>
+      </c>
+      <c r="X12" s="2" t="n">
+        <v>42.187</v>
+      </c>
+      <c r="Y12" s="2" t="n">
+        <v>33.768</v>
+      </c>
+      <c r="Z12" s="2" t="inlineStr">
+        <is>
+          <t>split</t>
+        </is>
+      </c>
+      <c r="AA12" s="2" t="inlineStr">
+        <is>
+          <t>measured</t>
+        </is>
+      </c>
+      <c r="AB12" s="2" t="inlineStr">
+        <is>
+          <t>multi_x5_329MHz.csv (sparse_4x4_x5_375_split.xclbin)</t>
+        </is>
+      </c>
+      <c r="AC12" s="2" t="inlineStr">
+        <is>
+          <t>steady state: sum over tenants of MACs / (active span - a), all tenants running; energy = full-set MIXED soak power / that</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>3 x 8x4 (30 ch)</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="n">
+        <v>66.795</v>
+      </c>
+      <c r="F13" s="2" t="n">
+        <v>0.5106000000000001</v>
+      </c>
+      <c r="G13" s="2" t="n">
+        <v>0.1409</v>
+      </c>
+      <c r="I13" s="2" t="n">
+        <v>354</v>
+      </c>
+      <c r="K13" s="2" t="n">
+        <v>2.2265</v>
+      </c>
+      <c r="L13" s="2" t="inlineStr">
+        <is>
+          <t>multi-tenant</t>
+        </is>
+      </c>
+      <c r="M13" s="2" t="inlineStr">
+        <is>
+          <t>3 x 8x4 tenants</t>
+        </is>
+      </c>
+      <c r="N13" s="2" t="inlineStr">
+        <is>
+          <t>8x4</t>
+        </is>
+      </c>
+      <c r="O13" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="P13" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="Q13" s="2" t="n">
+        <v>96</v>
+      </c>
+      <c r="R13" s="2" t="n">
+        <v>192</v>
+      </c>
+      <c r="S13" s="2" t="n">
+        <v>354</v>
+      </c>
+      <c r="T13" s="2" t="n">
+        <v>66.795</v>
+      </c>
+      <c r="U13" s="2" t="n">
+        <v>98.27</v>
+      </c>
+      <c r="V13" s="2" t="n">
+        <v>2.2265</v>
+      </c>
+      <c r="W13" s="2" t="n">
+        <v>0.6515</v>
+      </c>
+      <c r="X13" s="2" t="n">
+        <v>43.516</v>
+      </c>
+      <c r="Y13" s="2" t="n">
+        <v>34.106</v>
+      </c>
+      <c r="Z13" s="2" t="inlineStr">
+        <is>
+          <t>split</t>
+        </is>
+      </c>
+      <c r="AA13" s="2" t="inlineStr">
+        <is>
+          <t>measured</t>
+        </is>
+      </c>
+      <c r="AB13" s="2" t="inlineStr">
+        <is>
+          <t>multi_8x4_x3_354MHz.csv (sparse_8x4_x3_375.xclbin)</t>
+        </is>
+      </c>
+      <c r="AC13" s="2" t="inlineStr">
+        <is>
+          <t>steady state: sum over tenants of MACs / (active span - a), all tenants running; energy = full-set MIXED soak power / that</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>4x32 (32 ch)</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="n">
+        <v>63.635</v>
+      </c>
+      <c r="D14" s="2" t="n">
+        <v>0.5294</v>
+      </c>
+      <c r="E14" s="2" t="n">
+        <v>0.1349</v>
+      </c>
+      <c r="H14" s="2" t="n">
+        <v>250</v>
+      </c>
+      <c r="J14" s="2" t="n">
+        <v>1.9886</v>
+      </c>
+      <c r="L14" s="2" t="inlineStr">
+        <is>
+          <t>single engine</t>
+        </is>
+      </c>
+      <c r="M14" s="2" t="inlineStr">
+        <is>
+          <t>one 4x32 engine</t>
+        </is>
+      </c>
+      <c r="N14" s="2" t="inlineStr">
+        <is>
+          <t>4x32</t>
+        </is>
+      </c>
+      <c r="O14" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="P14" s="2" t="n">
+        <v>32</v>
+      </c>
+      <c r="Q14" s="2" t="n">
+        <v>128</v>
+      </c>
+      <c r="R14" s="2" t="n">
+        <v>256</v>
+      </c>
+      <c r="S14" s="2" t="n">
+        <v>250</v>
+      </c>
+      <c r="T14" s="2" t="n">
+        <v>63.635</v>
+      </c>
+      <c r="U14" s="2" t="n">
+        <v>99.43000000000001</v>
+      </c>
+      <c r="V14" s="2" t="n">
+        <v>1.9886</v>
+      </c>
+      <c r="W14" s="2" t="n">
+        <v>0.6643</v>
+      </c>
+      <c r="X14" s="2" t="n">
+        <v>42.271</v>
+      </c>
+      <c r="Y14" s="2" t="n">
+        <v>33.686</v>
+      </c>
+      <c r="Z14" s="2" t="inlineStr">
+        <is>
+          <t>split</t>
+        </is>
+      </c>
+      <c r="AA14" s="2" t="inlineStr">
+        <is>
+          <t>measured</t>
+        </is>
+      </c>
+      <c r="AB14" s="2" t="inlineStr">
+        <is>
+          <t>GEMV_Family_Measured.csv, family_measurements/4x32/power_4x32_250MHz.csv</t>
+        </is>
+      </c>
+      <c r="AC14" s="2" t="inlineStr">
+        <is>
+          <t>steady state: ss_gflops_act_MIXED / 2; energy = MIXED soak power / that</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:AC14"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>